<commit_message>
docs: refresh inference revision evidence
</commit_message>
<xml_diff>
--- a/docs/yolo_inference_RevisionNote.xlsx
+++ b/docs/yolo_inference_RevisionNote.xlsx
@@ -12,19 +12,25 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Evidence" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Engineering Log'!$A$5:$I$23</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Project Overview'!$A$1:$C$26</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Release Summary'!$A$1:$D$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Engineering Log'!$A$5:$I$25</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Engineering Log'!$1:$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Validation Evidence'!$A$4:$J$11</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Engineering Log'!$A$1:$I$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Validation Evidence'!$A$4:$J$16</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Validation Evidence'!$1:$4</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Validation Evidence'!$A$1:$J$16</definedName>
   </definedNames>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="17">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
+  <fonts count="18">
     <font>
       <name val="新細明體"/>
       <charset val="136"/>
@@ -134,8 +140,14 @@
       <color rgb="001F4E78"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -171,6 +183,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4B183"/>
       </patternFill>
     </fill>
   </fills>
@@ -343,7 +360,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -532,6 +549,18 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -641,8 +670,7 @@
     </comment>
     <comment ref="F9" authorId="0" shapeId="0">
       <text>
-        <t>Exact recorded command / activity:
-python -m pytest &lt;targeted suite&gt;</t>
+        <t>Legacy evidence provenance is incomplete. The prior placeholder command was removed; the exact executable, full pytest command, commit, timestamp, and log artifact were not recorded. Do not treat this row as reproducible CI evidence.</t>
       </text>
     </comment>
     <comment ref="F10" authorId="0" shapeId="0">
@@ -655,6 +683,46 @@
       <text>
         <t>Exact recorded command / activity:
 python -m pytest test_system_version test_fusion_inference test_result_handler test_light_controller test_light_handler test_auto_inspection_controller_lifecycle test_runtime_manifest</t>
+      </text>
+    </comment>
+    <comment ref="F12" authorId="0" shapeId="0">
+      <text>
+        <t>Historical targeted run dated 2026-08-13. Exact executable, full command, commit, timestamp, and log artifact were not recorded in the source revision note. Provenance remains incomplete; do not infer more than the displayed count.</t>
+      </text>
+    </comment>
+    <comment ref="F13" authorId="0" shapeId="0">
+      <text>
+        <t>Historical full-suite run dated 2026-08-13. Exact executable, full command, commit, timestamp, and log artifact were not recorded. The run was blocked by the documented host disk-capacity guard and is not a PASS.</t>
+      </text>
+    </comment>
+    <comment ref="F14" authorId="0" shapeId="0">
+      <text>
+        <t>Repository: https://github.com/DioWang67/Yolo_anomalib
+Evidence subject (tested code baseline): 8582a8b0a1c39d1ef4f27a1208a73f4e0c201cec
+Execution date: 2026-08-19; exact timestamps and runner paths are in the linked logs.
+Job commands: python -m ruff ...; python -m mypy ...; python -m pytest -m 'not gui' --timeout=60; python -m pytest -m gui --timeout=60; coverage gates; call build_exe.bat.
+PR CI/logs: https://github.com/DioWang67/Yolo_anomalib/actions/runs/32205343878
+Windows EXE/artifact log: https://github.com/DioWang67/Yolo_anomalib/actions/runs/32205366029</t>
+      </text>
+    </comment>
+    <comment ref="F15" authorId="0" shapeId="0">
+      <text>
+        <t>Repository: https://github.com/DioWang67/Yolo11_auto_train
+Exact SHA: 41589fc86b09311e885a8ba73c644728b6e00556
+Execution date: 2026-08-19; exact timestamps and runner paths are in the linked logs.
+Job commands: python -m ruff check src tests; python -m mypy src/picture_tool; python -m pytest --ignore=src/picture_tool/libs/labelImg --timeout=60; coverage and package build gates.
+Push CI/logs: https://github.com/DioWang67/Yolo11_auto_train/actions/runs/32205326796
+PR CI/logs: https://github.com/DioWang67/Yolo11_auto_train/actions/runs/32205329324</t>
+      </text>
+    </comment>
+    <comment ref="F16" authorId="0" shapeId="0">
+      <text>
+        <t>Repository: https://github.com/DioWang67/Yolo11_workspace
+Evidence subject (pre-document integration baseline): ee883171ce3732be486f5ac554a3c96d116bc969
+Execution date: 2026-08-19; exact timestamps and runner paths are in the linked logs.
+Job commands: python scripts/verify_submodule_checks.py --root .; python scripts/validate_workspace.py --root .; python -m pytest -q tests --cov=scripts --cov-fail-under=80; pinned child workspace-path tests.
+Push CI/logs: https://github.com/DioWang67/Yolo11_workspace/actions/runs/32206682344
+PR CI/logs: https://github.com/DioWang67/Yolo11_workspace/actions/runs/32206684956</t>
       </text>
     </comment>
   </commentList>
@@ -694,53 +762,6 @@
         <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="66675" y="9525"/>
           <a:ext cx="2076450" cy="790575"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-          <a:headEnd/>
-          <a:tailEnd/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>66675</colOff>
-      <row>0</row>
-      <rowOff>9525</rowOff>
-    </from>
-    <to>
-      <col>2</col>
-      <colOff>1346200</colOff>
-      <row>1</row>
-      <rowOff>0</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="4" name="Picture 12" descr="標準logo應用版"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeArrowheads="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" l="3822"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr bwMode="auto">
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="66675" y="9525"/>
-          <a:ext cx="2441575" cy="790575"/>
         </a:xfrm>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
@@ -1103,7 +1124,7 @@
     <row r="2" ht="24" customHeight="1" s="41">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Project Overview ? Formal Software Baseline v1.1.0</t>
+          <t>Project Overview — Documented Software Baseline v1.1.0</t>
         </is>
       </c>
     </row>
@@ -1175,10 +1196,10 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="32" customHeight="1" s="41">
+    <row r="8" ht="55" customHeight="1" s="41">
       <c r="A8" s="46" t="inlineStr">
         <is>
-          <t>Current Version</t>
+          <t>Documented Baseline Version</t>
         </is>
       </c>
       <c r="B8" s="47" t="inlineStr">
@@ -1188,24 +1209,22 @@
       </c>
       <c r="C8" s="47" t="inlineStr">
         <is>
-          <t>Backward-compatible minor release on the v1.0.0 baseline. Git tag and release package are still pending.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="32" customHeight="1" s="41">
+          <t>v1.1.0 remains the documented MINOR baseline because it introduced externally observable machine-readable inspection status contracts. The current merge candidate is Unreleased; no immutable tag or formal package has been issued.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1" s="41">
       <c r="A9" s="46" t="inlineStr">
         <is>
-          <t>Formal Release Date</t>
-        </is>
-      </c>
-      <c r="B9" s="47" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
+          <t>Baseline Documentation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="59" t="n">
+        <v>46247</v>
       </c>
       <c r="C9" s="47" t="inlineStr">
         <is>
-          <t>Software release date, not production-line acceptance date.</t>
+          <t>Documentation date only; not evidence of a tagged package or production acceptance.</t>
         </is>
       </c>
     </row>
@@ -1217,7 +1236,7 @@
       </c>
       <c r="B10" s="47" t="inlineStr">
         <is>
-          <t>2025/12 ? 2026/08</t>
+          <t>2025/12–2026/08</t>
         </is>
       </c>
       <c r="C10" s="47" t="inlineStr">
@@ -1234,7 +1253,7 @@
       </c>
       <c r="B11" s="47" t="inlineStr">
         <is>
-          <t>Python 3.10?3.11</t>
+          <t>Python 3.10–3.11</t>
         </is>
       </c>
       <c r="C11" s="47" t="inlineStr">
@@ -1302,7 +1321,7 @@
       </c>
       <c r="B15" s="47" t="inlineStr">
         <is>
-          <t>SQLite ? inspection_records.sqlite3</t>
+          <t>SQLite — inspection_records.sqlite3</t>
         </is>
       </c>
       <c r="C15" s="47" t="inlineStr">
@@ -1379,7 +1398,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="32" customHeight="1" s="41">
+    <row r="20" ht="58" customHeight="1" s="41">
       <c r="A20" s="46" t="inlineStr">
         <is>
           <t>Validation Status</t>
@@ -1387,16 +1406,16 @@
       </c>
       <c r="B20" s="47" t="inlineStr">
         <is>
-          <t>Targeted automated regression recorded; physical line validation pending</t>
+          <t>Exact-SHA automated checks passed; field acceptance remains pending</t>
         </is>
       </c>
       <c r="C20" s="47" t="inlineStr">
         <is>
-          <t>Earlier runs: 381 passed / 2 skipped. Formal baseline: 45 passed. v1.1.0: 192 targeted passed; full suite 1591 passed with 12 host disk-capacity failures also present on an unmodified baseline. Runs overlap and are not a coverage report.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="32" customHeight="1" s="41">
+          <t>Inference 8582a8b, Training 41589fc, and Workspace ee88317 CI passed. Inference workflow_dispatch also built and verified the Windows executable. These runs overlap and do not certify production-line operation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="58" customHeight="1" s="41">
       <c r="A21" s="46" t="inlineStr">
         <is>
           <t>Release Boundary</t>
@@ -1404,12 +1423,12 @@
       </c>
       <c r="B21" s="47" t="inlineStr">
         <is>
-          <t>Formal software release ? production certification</t>
+          <t>Code-only integration under report_only ≠ production suppress activation</t>
         </is>
       </c>
       <c r="C21" s="47" t="inlineStr">
         <is>
-          <t>Camera endurance, PLC, server sync, latency percentiles, and product accuracy remain separate gates.</t>
+          <t>Cable1/A remains report_only. A current-head camera cycle, one complete shift and at least 500 cycles, sync/retention/rollback evidence, and named approvals are required before suppress is enabled.</t>
         </is>
       </c>
     </row>
@@ -1469,7 +1488,7 @@
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1477,9 +1496,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BE26"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.2"/>
   <cols>
     <col width="15" customWidth="1" style="27" min="1" max="1"/>
@@ -1492,30 +1511,6 @@
   <sheetData>
     <row r="1" ht="63" customFormat="1" customHeight="1" s="7">
       <c r="A1" s="3" t="n"/>
-      <c r="L1" s="4" t="n"/>
-      <c r="M1" s="4" t="n"/>
-      <c r="N1" s="5" t="n"/>
-      <c r="O1" s="5" t="n"/>
-      <c r="P1" s="5" t="n"/>
-      <c r="Q1" s="6" t="n"/>
-      <c r="R1" s="4" t="n"/>
-      <c r="S1" s="4" t="n"/>
-      <c r="T1" s="5" t="n"/>
-      <c r="U1" s="5" t="n"/>
-      <c r="V1" s="5" t="n"/>
-      <c r="W1" s="6" t="n"/>
-      <c r="X1" s="4" t="n"/>
-      <c r="Y1" s="4" t="n"/>
-      <c r="Z1" s="5" t="n"/>
-      <c r="AA1" s="5" t="n"/>
-      <c r="AB1" s="5" t="n"/>
-      <c r="AC1" s="6" t="n"/>
-      <c r="AD1" s="4" t="n"/>
-      <c r="AE1" s="4" t="n"/>
-      <c r="AF1" s="5" t="n"/>
-      <c r="AG1" s="5" t="n"/>
-      <c r="AH1" s="5" t="n"/>
-      <c r="AI1" s="6" t="n"/>
     </row>
     <row r="2" ht="16.5" customFormat="1" customHeight="1" s="10">
       <c r="A2" s="38" t="inlineStr">
@@ -1526,59 +1521,6 @@
       <c r="B2" s="39" t="n"/>
       <c r="C2" s="39" t="n"/>
       <c r="D2" s="39" t="n"/>
-      <c r="E2" s="31" t="n"/>
-      <c r="F2" s="31" t="n"/>
-      <c r="G2" s="8" t="n"/>
-      <c r="H2" s="8" t="n"/>
-      <c r="I2" s="8" t="n"/>
-      <c r="J2" s="8" t="n"/>
-      <c r="K2" s="8" t="n"/>
-      <c r="L2" s="32" t="n"/>
-      <c r="M2" s="33" t="n"/>
-      <c r="N2" s="33" t="n"/>
-      <c r="O2" s="33" t="n"/>
-      <c r="P2" s="33" t="n"/>
-      <c r="Q2" s="34" t="n"/>
-      <c r="R2" s="32" t="n"/>
-      <c r="S2" s="33" t="n"/>
-      <c r="T2" s="33" t="n"/>
-      <c r="U2" s="33" t="n"/>
-      <c r="V2" s="33" t="n"/>
-      <c r="W2" s="34" t="n"/>
-      <c r="X2" s="32" t="n"/>
-      <c r="Y2" s="33" t="n"/>
-      <c r="Z2" s="33" t="n"/>
-      <c r="AA2" s="33" t="n"/>
-      <c r="AB2" s="33" t="n"/>
-      <c r="AC2" s="34" t="n"/>
-      <c r="AD2" s="32" t="n"/>
-      <c r="AE2" s="33" t="n"/>
-      <c r="AF2" s="33" t="n"/>
-      <c r="AG2" s="33" t="n"/>
-      <c r="AH2" s="33" t="n"/>
-      <c r="AI2" s="34" t="n"/>
-      <c r="AJ2" s="9" t="n"/>
-      <c r="AK2" s="9" t="n"/>
-      <c r="AL2" s="9" t="n"/>
-      <c r="AM2" s="9" t="n"/>
-      <c r="AN2" s="9" t="n"/>
-      <c r="AO2" s="9" t="n"/>
-      <c r="AP2" s="9" t="n"/>
-      <c r="AQ2" s="9" t="n"/>
-      <c r="AR2" s="9" t="n"/>
-      <c r="AS2" s="9" t="n"/>
-      <c r="AT2" s="9" t="n"/>
-      <c r="AU2" s="9" t="n"/>
-      <c r="AV2" s="9" t="n"/>
-      <c r="AW2" s="9" t="n"/>
-      <c r="AX2" s="9" t="n"/>
-      <c r="AY2" s="9" t="n"/>
-      <c r="AZ2" s="9" t="n"/>
-      <c r="BA2" s="9" t="n"/>
-      <c r="BB2" s="9" t="n"/>
-      <c r="BC2" s="9" t="n"/>
-      <c r="BD2" s="9" t="n"/>
-      <c r="BE2" s="9" t="n"/>
     </row>
     <row r="3" ht="16.5" customFormat="1" customHeight="1" s="10">
       <c r="A3" s="38" t="inlineStr">
@@ -1589,201 +1531,33 @@
       <c r="B3" s="39" t="n"/>
       <c r="C3" s="39" t="n"/>
       <c r="D3" s="39" t="n"/>
-      <c r="E3" s="12" t="n"/>
-      <c r="F3" s="12" t="n"/>
-      <c r="G3" s="8" t="n"/>
-      <c r="H3" s="8" t="n"/>
-      <c r="I3" s="8" t="n"/>
-      <c r="J3" s="8" t="n"/>
-      <c r="K3" s="8" t="n"/>
-      <c r="L3" s="32" t="n"/>
-      <c r="M3" s="33" t="n"/>
-      <c r="N3" s="33" t="n"/>
-      <c r="O3" s="33" t="n"/>
-      <c r="P3" s="33" t="n"/>
-      <c r="Q3" s="34" t="n"/>
-      <c r="R3" s="32" t="n"/>
-      <c r="S3" s="33" t="n"/>
-      <c r="T3" s="33" t="n"/>
-      <c r="U3" s="33" t="n"/>
-      <c r="V3" s="33" t="n"/>
-      <c r="W3" s="34" t="n"/>
-      <c r="X3" s="32" t="n"/>
-      <c r="Y3" s="33" t="n"/>
-      <c r="Z3" s="33" t="n"/>
-      <c r="AA3" s="33" t="n"/>
-      <c r="AB3" s="33" t="n"/>
-      <c r="AC3" s="34" t="n"/>
-      <c r="AD3" s="32" t="n"/>
-      <c r="AE3" s="33" t="n"/>
-      <c r="AF3" s="33" t="n"/>
-      <c r="AG3" s="33" t="n"/>
-      <c r="AH3" s="33" t="n"/>
-      <c r="AI3" s="34" t="n"/>
-      <c r="AJ3" s="9" t="n"/>
-      <c r="AK3" s="9" t="n"/>
-      <c r="AL3" s="9" t="n"/>
-      <c r="AM3" s="9" t="n"/>
-      <c r="AN3" s="9" t="n"/>
-      <c r="AO3" s="9" t="n"/>
-      <c r="AP3" s="9" t="n"/>
-      <c r="AQ3" s="9" t="n"/>
-      <c r="AR3" s="9" t="n"/>
-      <c r="AS3" s="9" t="n"/>
-      <c r="AT3" s="9" t="n"/>
-      <c r="AU3" s="9" t="n"/>
-      <c r="AV3" s="9" t="n"/>
-      <c r="AW3" s="9" t="n"/>
-      <c r="AX3" s="9" t="n"/>
-      <c r="AY3" s="9" t="n"/>
-      <c r="AZ3" s="9" t="n"/>
-      <c r="BA3" s="9" t="n"/>
-      <c r="BB3" s="9" t="n"/>
-      <c r="BC3" s="9" t="n"/>
-      <c r="BD3" s="9" t="n"/>
-      <c r="BE3" s="9" t="n"/>
     </row>
     <row r="4" ht="16.5" customFormat="1" customHeight="1" s="18">
       <c r="A4" s="40" t="inlineStr">
         <is>
-          <t>Design Responsibility : DioWang</t>
+          <t>Design Responsibility : Dio Wang</t>
         </is>
       </c>
       <c r="B4" s="33" t="n"/>
       <c r="C4" s="34" t="n"/>
       <c r="D4" s="11" t="n"/>
-      <c r="E4" s="12" t="n"/>
-      <c r="F4" s="12" t="n"/>
-      <c r="G4" s="12" t="n"/>
-      <c r="H4" s="12" t="n"/>
-      <c r="I4" s="12" t="n"/>
-      <c r="J4" s="13" t="n"/>
-      <c r="K4" s="37" t="n"/>
-      <c r="L4" s="33" t="n"/>
-      <c r="M4" s="34" t="n"/>
-      <c r="N4" s="14" t="n"/>
-      <c r="O4" s="14" t="n"/>
-      <c r="P4" s="14" t="n"/>
-      <c r="Q4" s="15" t="n"/>
-      <c r="R4" s="16" t="n"/>
-      <c r="S4" s="14" t="n"/>
-      <c r="T4" s="14" t="n"/>
-      <c r="U4" s="14" t="n"/>
-      <c r="V4" s="14" t="n"/>
-      <c r="W4" s="15" t="n"/>
-      <c r="X4" s="16" t="n"/>
-      <c r="Y4" s="14" t="n"/>
-      <c r="Z4" s="14" t="n"/>
-      <c r="AA4" s="14" t="n"/>
-      <c r="AB4" s="14" t="n"/>
-      <c r="AC4" s="15" t="n"/>
-      <c r="AD4" s="16" t="n"/>
-      <c r="AE4" s="14" t="n"/>
-      <c r="AF4" s="14" t="n"/>
-      <c r="AG4" s="14" t="n"/>
-      <c r="AH4" s="14" t="n"/>
-      <c r="AI4" s="15" t="n"/>
-      <c r="AJ4" s="17" t="n"/>
-      <c r="AK4" s="17" t="n"/>
-      <c r="AL4" s="17" t="n"/>
-      <c r="AM4" s="17" t="n"/>
-      <c r="AN4" s="17" t="n"/>
-      <c r="AO4" s="17" t="n"/>
-      <c r="AP4" s="17" t="n"/>
-      <c r="AQ4" s="17" t="n"/>
-      <c r="AR4" s="17" t="n"/>
-      <c r="AS4" s="17" t="n"/>
-      <c r="AT4" s="17" t="n"/>
-      <c r="AU4" s="17" t="n"/>
-      <c r="AV4" s="17" t="n"/>
-      <c r="AW4" s="17" t="n"/>
-      <c r="AX4" s="17" t="n"/>
-      <c r="AY4" s="17" t="n"/>
-      <c r="AZ4" s="17" t="n"/>
-      <c r="BA4" s="17" t="n"/>
-      <c r="BB4" s="17" t="n"/>
-      <c r="BC4" s="17" t="n"/>
-      <c r="BD4" s="17" t="n"/>
-      <c r="BE4" s="17" t="n"/>
     </row>
     <row r="5" ht="16.5" customFormat="1" customHeight="1" s="17">
       <c r="A5" s="35" t="inlineStr">
         <is>
-          <t>Prepared By : DioWang</t>
+          <t>Prepared By : Dio Wang</t>
         </is>
       </c>
       <c r="B5" s="36" t="n"/>
       <c r="C5" s="36" t="n"/>
       <c r="D5" s="30" t="inlineStr">
         <is>
-          <t>Release Date :  2026 / 08 / 13</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="n"/>
-      <c r="F5" s="2" t="n"/>
-      <c r="G5" s="20" t="n"/>
-      <c r="H5" s="20" t="n"/>
-      <c r="I5" s="20" t="n"/>
-      <c r="J5" s="20" t="n"/>
-      <c r="K5" s="21" t="n"/>
-      <c r="L5" s="22" t="n"/>
-      <c r="M5" s="22" t="n"/>
-      <c r="N5" s="23" t="n"/>
-      <c r="O5" s="23" t="n"/>
-      <c r="P5" s="23" t="n"/>
-      <c r="Q5" s="24" t="n"/>
-      <c r="R5" s="23" t="n"/>
-      <c r="S5" s="23" t="n"/>
-      <c r="T5" s="23" t="n"/>
-      <c r="U5" s="23" t="n"/>
-      <c r="V5" s="23" t="n"/>
-      <c r="W5" s="24" t="n"/>
-      <c r="X5" s="23" t="n"/>
-      <c r="Y5" s="23" t="n"/>
-      <c r="Z5" s="23" t="n"/>
-      <c r="AA5" s="23" t="n"/>
-      <c r="AB5" s="23" t="n"/>
-      <c r="AC5" s="24" t="n"/>
-      <c r="AD5" s="23" t="n"/>
-      <c r="AE5" s="23" t="n"/>
-      <c r="AF5" s="23" t="n"/>
-      <c r="AG5" s="23" t="n"/>
-      <c r="AH5" s="23" t="n"/>
-      <c r="AI5" s="24" t="n"/>
+          <t>Baseline Date : 2026-08-13</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="16.5" customFormat="1" customHeight="1" s="17">
       <c r="D6" s="19" t="n"/>
-      <c r="E6" s="20" t="n"/>
-      <c r="F6" s="20" t="n"/>
-      <c r="G6" s="20" t="n"/>
-      <c r="H6" s="20" t="n"/>
-      <c r="I6" s="20" t="n"/>
-      <c r="J6" s="20" t="n"/>
-      <c r="K6" s="21" t="n"/>
-      <c r="L6" s="22" t="n"/>
-      <c r="M6" s="22" t="n"/>
-      <c r="N6" s="23" t="n"/>
-      <c r="O6" s="23" t="n"/>
-      <c r="P6" s="23" t="n"/>
-      <c r="Q6" s="24" t="n"/>
-      <c r="R6" s="23" t="n"/>
-      <c r="S6" s="23" t="n"/>
-      <c r="T6" s="23" t="n"/>
-      <c r="U6" s="23" t="n"/>
-      <c r="V6" s="23" t="n"/>
-      <c r="W6" s="24" t="n"/>
-      <c r="X6" s="23" t="n"/>
-      <c r="Y6" s="23" t="n"/>
-      <c r="Z6" s="23" t="n"/>
-      <c r="AA6" s="23" t="n"/>
-      <c r="AB6" s="23" t="n"/>
-      <c r="AC6" s="24" t="n"/>
-      <c r="AD6" s="23" t="n"/>
-      <c r="AE6" s="23" t="n"/>
-      <c r="AF6" s="23" t="n"/>
-      <c r="AG6" s="23" t="n"/>
-      <c r="AH6" s="23" t="n"/>
-      <c r="AI6" s="24" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="25" t="inlineStr">
@@ -1803,15 +1577,13 @@
       </c>
       <c r="D7" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Description </t>
+          <t>Description</t>
         </is>
       </c>
     </row>
     <row r="8" ht="55.2" customHeight="1" s="41">
-      <c r="A8" s="28" t="inlineStr">
-        <is>
-          <t>12/19/2025</t>
-        </is>
+      <c r="A8" s="60" t="n">
+        <v>46010</v>
       </c>
       <c r="B8" s="29" t="inlineStr">
         <is>
@@ -1830,10 +1602,8 @@
       </c>
     </row>
     <row r="9" ht="55.2" customHeight="1" s="41">
-      <c r="A9" s="28" t="inlineStr">
-        <is>
-          <t>1/7/2026</t>
-        </is>
+      <c r="A9" s="60" t="n">
+        <v>46029</v>
       </c>
       <c r="B9" s="29" t="inlineStr">
         <is>
@@ -1852,10 +1622,8 @@
       </c>
     </row>
     <row r="10" ht="55.2" customHeight="1" s="41">
-      <c r="A10" s="28" t="inlineStr">
-        <is>
-          <t>1/15/2026</t>
-        </is>
+      <c r="A10" s="60" t="n">
+        <v>46037</v>
       </c>
       <c r="B10" s="29" t="inlineStr">
         <is>
@@ -1874,10 +1642,8 @@
       </c>
     </row>
     <row r="11" ht="55.2" customHeight="1" s="41">
-      <c r="A11" s="28" t="inlineStr">
-        <is>
-          <t>2/11/2026</t>
-        </is>
+      <c r="A11" s="60" t="n">
+        <v>46064</v>
       </c>
       <c r="B11" s="29" t="inlineStr">
         <is>
@@ -1896,10 +1662,8 @@
       </c>
     </row>
     <row r="12" ht="55.2" customHeight="1" s="41">
-      <c r="A12" s="28" t="inlineStr">
-        <is>
-          <t>3/11/2026</t>
-        </is>
+      <c r="A12" s="60" t="n">
+        <v>46092</v>
       </c>
       <c r="B12" s="29" t="inlineStr">
         <is>
@@ -1913,15 +1677,13 @@
       </c>
       <c r="D12" s="29" t="inlineStr">
         <is>
-          <t>Replaced broad exception handling, corrected configuration / result contracts, fixed pytest crashes, and restored Ruff and strict MyPy checks without adding a new operator workflow.</t>
+          <t>Replaced broad exception handling, corrected configuration / result contracts, fixed pytest crashes, and restored Ruff and configured scoped mypy CI checks without adding a new operator workflow.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="55.2" customHeight="1" s="41">
-      <c r="A13" s="28" t="inlineStr">
-        <is>
-          <t>3/30/2026</t>
-        </is>
+      <c r="A13" s="60" t="n">
+        <v>46111</v>
       </c>
       <c r="B13" s="29" t="inlineStr">
         <is>
@@ -1940,10 +1702,8 @@
       </c>
     </row>
     <row r="14" ht="55.2" customHeight="1" s="41">
-      <c r="A14" s="28" t="inlineStr">
-        <is>
-          <t>3/31/2026</t>
-        </is>
+      <c r="A14" s="60" t="n">
+        <v>46112</v>
       </c>
       <c r="B14" s="29" t="inlineStr">
         <is>
@@ -1962,10 +1722,8 @@
       </c>
     </row>
     <row r="15" ht="55.2" customHeight="1" s="41">
-      <c r="A15" s="28" t="inlineStr">
-        <is>
-          <t>5/28/2026</t>
-        </is>
+      <c r="A15" s="60" t="n">
+        <v>46170</v>
       </c>
       <c r="B15" s="29" t="inlineStr">
         <is>
@@ -1984,10 +1742,8 @@
       </c>
     </row>
     <row r="16" ht="55.2" customHeight="1" s="41">
-      <c r="A16" s="28" t="inlineStr">
-        <is>
-          <t>6/11/2026</t>
-        </is>
+      <c r="A16" s="60" t="n">
+        <v>46184</v>
       </c>
       <c r="B16" s="29" t="inlineStr">
         <is>
@@ -2006,10 +1762,8 @@
       </c>
     </row>
     <row r="17" ht="55.2" customHeight="1" s="41">
-      <c r="A17" s="28" t="inlineStr">
-        <is>
-          <t>6/25/2026</t>
-        </is>
+      <c r="A17" s="60" t="n">
+        <v>46198</v>
       </c>
       <c r="B17" s="29" t="inlineStr">
         <is>
@@ -2028,10 +1782,8 @@
       </c>
     </row>
     <row r="18" ht="55.2" customHeight="1" s="41">
-      <c r="A18" s="28" t="inlineStr">
-        <is>
-          <t>6/30/2026</t>
-        </is>
+      <c r="A18" s="60" t="n">
+        <v>46203</v>
       </c>
       <c r="B18" s="29" t="inlineStr">
         <is>
@@ -2050,10 +1802,8 @@
       </c>
     </row>
     <row r="19" ht="55.2" customHeight="1" s="41">
-      <c r="A19" s="28" t="inlineStr">
-        <is>
-          <t>7/9/2026</t>
-        </is>
+      <c r="A19" s="60" t="n">
+        <v>46212</v>
       </c>
       <c r="B19" s="29" t="inlineStr">
         <is>
@@ -2072,10 +1822,8 @@
       </c>
     </row>
     <row r="20" ht="55.2" customHeight="1" s="41">
-      <c r="A20" s="28" t="inlineStr">
-        <is>
-          <t>7/13/2026</t>
-        </is>
+      <c r="A20" s="60" t="n">
+        <v>46216</v>
       </c>
       <c r="B20" s="29" t="inlineStr">
         <is>
@@ -2094,10 +1842,8 @@
       </c>
     </row>
     <row r="21" ht="55.2" customHeight="1" s="41">
-      <c r="A21" s="28" t="inlineStr">
-        <is>
-          <t>7/24/2026</t>
-        </is>
+      <c r="A21" s="60" t="n">
+        <v>46227</v>
       </c>
       <c r="B21" s="29" t="inlineStr">
         <is>
@@ -2116,10 +1862,8 @@
       </c>
     </row>
     <row r="22" ht="55.2" customHeight="1" s="41">
-      <c r="A22" s="28" t="inlineStr">
-        <is>
-          <t>7/30/2026</t>
-        </is>
+      <c r="A22" s="60" t="n">
+        <v>46233</v>
       </c>
       <c r="B22" s="29" t="inlineStr">
         <is>
@@ -2138,10 +1882,8 @@
       </c>
     </row>
     <row r="23" ht="55.2" customHeight="1" s="41">
-      <c r="A23" s="28" t="inlineStr">
-        <is>
-          <t>7/31/2026</t>
-        </is>
+      <c r="A23" s="60" t="n">
+        <v>46234</v>
       </c>
       <c r="B23" s="29" t="inlineStr">
         <is>
@@ -2160,10 +1902,8 @@
       </c>
     </row>
     <row r="24" ht="55.2" customHeight="1" s="41">
-      <c r="A24" s="28" t="inlineStr">
-        <is>
-          <t>8/3/2026</t>
-        </is>
+      <c r="A24" s="60" t="n">
+        <v>46237</v>
       </c>
       <c r="B24" s="29" t="inlineStr">
         <is>
@@ -2177,15 +1917,13 @@
       </c>
       <c r="D24" s="29" t="inlineStr">
         <is>
-          <t>`workspace.yaml` defines training, model, station, result, and release-artifact paths. Migration tools move mutable data out of source trees and preserve access to existing evidence around Windows file locks.</t>
+          <t>workspace.yaml defines training, model, station, result, and release-artifact paths. Migration tools move mutable data out of source trees and preserve access to existing evidence around Windows file locks.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="55.2" customHeight="1" s="41">
-      <c r="A25" s="28" t="inlineStr">
-        <is>
-          <t>8/5/2026</t>
-        </is>
+      <c r="A25" s="60" t="n">
+        <v>46239</v>
       </c>
       <c r="B25" s="29" t="inlineStr">
         <is>
@@ -2194,7 +1932,7 @@
       </c>
       <c r="C25" s="29" t="inlineStr">
         <is>
-          <t>First Formal Integrated Release</t>
+          <t>First Documented Integrated Baseline</t>
         </is>
       </c>
       <c r="D25" s="29" t="inlineStr">
@@ -2203,11 +1941,9 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="55.2" customHeight="1" s="41">
-      <c r="A26" s="28" t="inlineStr">
-        <is>
-          <t>8/13/2026</t>
-        </is>
+    <row r="26" ht="142" customHeight="1" s="41">
+      <c r="A26" s="60" t="n">
+        <v>46247</v>
       </c>
       <c r="B26" s="29" t="inlineStr">
         <is>
@@ -2221,28 +1957,39 @@
       </c>
       <c r="D26" s="29" t="inlineStr">
         <is>
-          <t>Color, count, and position checks that cannot be evaluated now fail the inspection instead of passing silently. An unreadable expected-items or position configuration, and a frame with no detection ROI, are recorded with an explicit status code rather than treated as nothing to check. Color checker runtime configuration is replaced on every invocation, so a checker reused across products cannot carry the previous product's thresholds into the next inspection.</t>
+          <t>Color, count, and position checks that cannot be evaluated now fail the inspection instead of passing silently. An unreadable expected-items or position configuration, and a frame with no detection ROI, are recorded with an explicit status code rather than treated as nothing to check. Color checker runtime configuration is replaced on every invocation, so a checker reused across products cannot carry the previous product's thresholds into the next inspection. Version 1.1.0 remains MINOR because the persisted machine-readable inspection status contract is an externally observable backward-compatible capability. Persisted triage-reason mapping for count/position configuration lookup failures and no-detection color cases remains incomplete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="108" customHeight="1" s="41">
+      <c r="A27" s="60" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B27" s="29" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="C27" s="29" t="inlineStr">
+        <is>
+          <t>Merge-Readiness and Report-Only Safety</t>
+        </is>
+      </c>
+      <c r="D27" s="29" t="inlineStr">
+        <is>
+          <t>Recorded crash-safe inspection release, rollback, and retention; fail-closed scoped pilot, preflight, and duplicate evidence; live-station test isolation; exact-SHA CI; and the Cable1/A report_only safety default. Verdicts remain fail-closed, but persisted triage-reason mapping is still incomplete for count/position configuration lookup and no-detection color cases. This is an integration entry, not a formal package or production certification.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="AD2:AI2"/>
-    <mergeCell ref="R2:W2"/>
-    <mergeCell ref="AD3:AI3"/>
+  <mergeCells count="4">
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="K4:M4"/>
-    <mergeCell ref="R3:W3"/>
+    <mergeCell ref="A4:C4"/>
     <mergeCell ref="A3:D3"/>
-    <mergeCell ref="X3:AC3"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="L3:Q3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="L2:Q2"/>
-    <mergeCell ref="X2:AC2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -2253,7 +2000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.2"/>
   <cols>
     <col width="13" customWidth="1" style="41" min="1" max="1"/>
@@ -2281,10 +2028,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="32" customHeight="1" s="41">
+    <row r="3" ht="52" customHeight="1" s="41">
       <c r="A3" s="44" t="inlineStr">
         <is>
-          <t>Recorded targeted runs: earlier suites reported 381 passed / 2 skipped; the v1.0.0 baseline suite reported 45 passed; the v1.1.0 run reported 192 targeted passed and a full suite of 1591 passed with 12 host disk-capacity failures. Runs overlap. No full coverage report or physical production-line validation was performed.</t>
+          <t>Recorded automated evidence now includes the v1.1.0 history and the 2026-08-19 exact-SHA GitHub checks: inference PR plus Windows executable, training push/PR, and workspace integration passed. Runs overlap; no current-head physical line validation, full-shift/500-cycle suppress pilot, or named operational approval is recorded.</t>
         </is>
       </c>
     </row>
@@ -2336,10 +2083,8 @@
       </c>
     </row>
     <row r="6" ht="190" customHeight="1" s="41">
-      <c r="A6" s="46" t="inlineStr">
-        <is>
-          <t>12/19/2025</t>
-        </is>
+      <c r="A6" s="61" t="n">
+        <v>46010</v>
       </c>
       <c r="B6" s="46" t="inlineStr">
         <is>
@@ -2389,10 +2134,8 @@
       </c>
     </row>
     <row r="7" ht="190" customHeight="1" s="41">
-      <c r="A7" s="46" t="inlineStr">
-        <is>
-          <t>1/7/2026</t>
-        </is>
+      <c r="A7" s="61" t="n">
+        <v>46029</v>
       </c>
       <c r="B7" s="46" t="inlineStr">
         <is>
@@ -2441,10 +2184,8 @@
       </c>
     </row>
     <row r="8" ht="190" customHeight="1" s="41">
-      <c r="A8" s="46" t="inlineStr">
-        <is>
-          <t>1/15/2026</t>
-        </is>
+      <c r="A8" s="61" t="n">
+        <v>46037</v>
       </c>
       <c r="B8" s="46" t="inlineStr">
         <is>
@@ -2495,10 +2236,8 @@
       </c>
     </row>
     <row r="9" ht="190" customHeight="1" s="41">
-      <c r="A9" s="46" t="inlineStr">
-        <is>
-          <t>2/11/2026</t>
-        </is>
+      <c r="A9" s="61" t="n">
+        <v>46064</v>
       </c>
       <c r="B9" s="46" t="inlineStr">
         <is>
@@ -2549,10 +2288,8 @@
       </c>
     </row>
     <row r="10" ht="190" customHeight="1" s="41">
-      <c r="A10" s="46" t="inlineStr">
-        <is>
-          <t>3/11/2026</t>
-        </is>
+      <c r="A10" s="61" t="n">
+        <v>46092</v>
       </c>
       <c r="B10" s="46" t="inlineStr">
         <is>
@@ -2571,7 +2308,7 @@
 - Corrected result and configuration boundaries.
 Test / CI changes
 - Fixed pytest collection / teardown failures.
-- Restored Ruff and strict MyPy checks and synchronized documentation.</t>
+- Restored Ruff and configured scoped mypy CI checks and synchronized documentation.</t>
         </is>
       </c>
       <c r="E10" s="47" t="inlineStr">
@@ -2603,10 +2340,8 @@
       </c>
     </row>
     <row r="11" ht="190" customHeight="1" s="41">
-      <c r="A11" s="46" t="inlineStr">
-        <is>
-          <t>3/30/2026</t>
-        </is>
+      <c r="A11" s="61" t="n">
+        <v>46111</v>
       </c>
       <c r="B11" s="46" t="inlineStr">
         <is>
@@ -2657,10 +2392,8 @@
       </c>
     </row>
     <row r="12" ht="190" customHeight="1" s="41">
-      <c r="A12" s="46" t="inlineStr">
-        <is>
-          <t>3/31/2026</t>
-        </is>
+      <c r="A12" s="61" t="n">
+        <v>46112</v>
       </c>
       <c r="B12" s="46" t="inlineStr">
         <is>
@@ -2708,10 +2441,8 @@
       </c>
     </row>
     <row r="13" ht="190" customHeight="1" s="41">
-      <c r="A13" s="46" t="inlineStr">
-        <is>
-          <t>5/28/2026</t>
-        </is>
+      <c r="A13" s="61" t="n">
+        <v>46170</v>
       </c>
       <c r="B13" s="46" t="inlineStr">
         <is>
@@ -2761,10 +2492,8 @@
       </c>
     </row>
     <row r="14" ht="190" customHeight="1" s="41">
-      <c r="A14" s="46" t="inlineStr">
-        <is>
-          <t>6/11/2026</t>
-        </is>
+      <c r="A14" s="61" t="n">
+        <v>46184</v>
       </c>
       <c r="B14" s="46" t="inlineStr">
         <is>
@@ -2813,10 +2542,8 @@
       </c>
     </row>
     <row r="15" ht="190" customHeight="1" s="41">
-      <c r="A15" s="46" t="inlineStr">
-        <is>
-          <t>6/25/2026</t>
-        </is>
+      <c r="A15" s="61" t="n">
+        <v>46198</v>
       </c>
       <c r="B15" s="46" t="inlineStr">
         <is>
@@ -2865,10 +2592,8 @@
       </c>
     </row>
     <row r="16" ht="190" customHeight="1" s="41">
-      <c r="A16" s="46" t="inlineStr">
-        <is>
-          <t>6/30/2026</t>
-        </is>
+      <c r="A16" s="61" t="n">
+        <v>46203</v>
       </c>
       <c r="B16" s="46" t="inlineStr">
         <is>
@@ -2914,10 +2639,8 @@
       </c>
     </row>
     <row r="17" ht="190" customHeight="1" s="41">
-      <c r="A17" s="46" t="inlineStr">
-        <is>
-          <t>7/9/2026</t>
-        </is>
+      <c r="A17" s="61" t="n">
+        <v>46212</v>
       </c>
       <c r="B17" s="46" t="inlineStr">
         <is>
@@ -2966,10 +2689,8 @@
       </c>
     </row>
     <row r="18" ht="190" customHeight="1" s="41">
-      <c r="A18" s="46" t="inlineStr">
-        <is>
-          <t>7/13/2026</t>
-        </is>
+      <c r="A18" s="61" t="n">
+        <v>46216</v>
       </c>
       <c r="B18" s="46" t="inlineStr">
         <is>
@@ -3016,10 +2737,8 @@
       </c>
     </row>
     <row r="19" ht="190" customHeight="1" s="41">
-      <c r="A19" s="46" t="inlineStr">
-        <is>
-          <t>7/24/2026</t>
-        </is>
+      <c r="A19" s="61" t="n">
+        <v>46227</v>
       </c>
       <c r="B19" s="46" t="inlineStr">
         <is>
@@ -3069,11 +2788,9 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="190" customHeight="1" s="41">
-      <c r="A20" s="46" t="inlineStr">
-        <is>
-          <t>7/30/2026</t>
-        </is>
+    <row r="20" ht="150" customHeight="1" s="41">
+      <c r="A20" s="61" t="n">
+        <v>46233</v>
       </c>
       <c r="B20" s="46" t="inlineStr">
         <is>
@@ -3082,17 +2799,16 @@
       </c>
       <c r="C20" s="47" t="inlineStr">
         <is>
-          <t>False rejects and missed detections were saved but not routed into a controlled correction / retraining path. Excel-only history was difficult to query, and deployment could pair an ONNX file with the wrong PT checkpoint.</t>
+          <t>The v0.8.0 correction workflow lacked searchable production history, dataset-conflict gates, position acceptance gates, and atomic ONNX/PT pairing.</t>
         </is>
       </c>
       <c r="D20" s="47" t="inlineStr">
         <is>
           <t>Core changes
-- Added review, annotation repair, batch preparation, and operator training screens.
-- Added stable sample IDs, dataset conflict checks, family-aware split checks, position Golden Set / Gate, and matching ONNX-PT deployment contracts.
-- Moved persistence off the inspection critical path.
-Supporting changes
-- Added SQLite inspections, ai_predictions, inspection_artifacts, review_events, maintenance_events, and inspection_sync_outbox tables.</t>
+- Added searchable SQLite inspection history and a synchronization outbox.
+- Added stable sample IDs and dataset-conflict checks.
+- Added position Golden Set / Gate evidence.
+- Added an atomic matching ONNX/PT deployment contract.</t>
         </is>
       </c>
       <c r="E20" s="47" t="inlineStr">
@@ -3124,10 +2840,8 @@
       </c>
     </row>
     <row r="21" ht="190" customHeight="1" s="41">
-      <c r="A21" s="46" t="inlineStr">
-        <is>
-          <t>7/31/2026</t>
-        </is>
+      <c r="A21" s="61" t="n">
+        <v>46234</v>
       </c>
       <c r="B21" s="46" t="inlineStr">
         <is>
@@ -3179,10 +2893,8 @@
       </c>
     </row>
     <row r="22" ht="190" customHeight="1" s="41">
-      <c r="A22" s="46" t="inlineStr">
-        <is>
-          <t>8/3/2026</t>
-        </is>
+      <c r="A22" s="61" t="n">
+        <v>46237</v>
       </c>
       <c r="B22" s="46" t="inlineStr">
         <is>
@@ -3235,10 +2947,8 @@
       </c>
     </row>
     <row r="23" ht="190" customHeight="1" s="41">
-      <c r="A23" s="46" t="inlineStr">
-        <is>
-          <t>8/5/2026</t>
-        </is>
+      <c r="A23" s="61" t="n">
+        <v>46239</v>
       </c>
       <c r="B23" s="46" t="inlineStr">
         <is>
@@ -3272,7 +2982,7 @@
       </c>
       <c r="G23" s="47" t="inlineStr">
         <is>
-          <t>Formal software release is not production-line certification. Physical camera endurance, PLC integration, server synchronization, latency percentiles, and product-specific accuracy acceptance remain separate gates. Git tag / release package is not created by this document update.</t>
+          <t>A documented software baseline is not production-line certification. Physical camera endurance, PLC integration, server synchronization, latency percentiles, and product-specific accuracy acceptance remain separate gates. An immutable Git tag / release package remains pending.</t>
         </is>
       </c>
       <c r="H23" s="47" t="inlineStr">
@@ -3286,11 +2996,9 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="190" customHeight="1" s="41">
-      <c r="A24" s="46" t="inlineStr">
-        <is>
-          <t>8/13/2026</t>
-        </is>
+    <row r="24" ht="292" customHeight="1" s="41">
+      <c r="A24" s="61" t="n">
+        <v>46247</v>
       </c>
       <c r="B24" s="46" t="inlineStr">
         <is>
@@ -3311,7 +3019,9 @@
 - finalize_status carries an unevaluable verdict through instead of re-deriving PASS from the absence of a signal.
 Supporting changes
 - Color checker runtime configuration is replaced, not merged, per invocation; invalid values raise instead of being silently discarded.
-- Operator text separates a color mismatch from a confidence shortfall across the verdict message, detail panel, and image overlay.</t>
+- Operator text separates a color mismatch from a confidence shortfall across the verdict message, detail panel, and image overlay.
+Versioning
+- Classified as MINOR because persisted machine-readable inspection status codes are an externally observable backward-compatible contract.</t>
         </is>
       </c>
       <c r="E24" s="47" t="inlineStr">
@@ -3324,7 +3034,7 @@
       </c>
       <c r="F24" s="47" t="inlineStr">
         <is>
-          <t>2026-08-13 targeted run: 192 passed across pipeline steps, color checker service, color result display, annotations, color override loader, and stats color checker. Full inference suite: 1591 passed, 1 skipped, 12 failed. The 12 failures are host disk-capacity guard trips in test_result_handler and were reproduced identically on an unmodified baseline. Ruff CI gate passed; MyPy findings on the touched modules went from 17 to 13.</t>
+          <t>2026-08-13 targeted run: 192 passed across pipeline steps, color checker service, color result display, annotations, color override loader, and stats color checker. Full inference suite: 1591 passed, 1 skipped, 12 failed. The 12 failures are host disk-capacity guard trips in test_result_handler and were reproduced identically on an unmodified baseline. Ruff CI gate passed. A separate non-blocking mypy audit of the v1.1.0-touched modules reported 13 remaining findings.</t>
         </is>
       </c>
       <c r="G24" s="47" t="inlineStr">
@@ -3344,15 +3054,69 @@
         </is>
       </c>
     </row>
+    <row r="25" ht="268" customHeight="1" s="41">
+      <c r="A25" s="61" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B25" s="46" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="C25" s="47" t="inlineStr">
+        <is>
+          <t>Release activation, validation, audit, and retention crossed mutable database, filesystem, and pointer boundaries. Pilot evidence could be incomplete or scoped to the wrong product/time window, tests could discover live station data, and Cable1/A suppression was not justified without the required field evidence.</t>
+        </is>
+      </c>
+      <c r="D25" s="47" t="inlineStr">
+        <is>
+          <t>Core changes
+- Made inspection release activation, rollback, audit linkage, and retention cleanup atomic or recoverable across process failures.
+- Added fail-closed, scope-bound pilot, preflight, and duplicate-audit evidence with immutable hashes.
+- Isolated pytest workspace discovery from live station data.
+- Set the tracked Cable1/A duplicate policy to report_only and added a regression guard.</t>
+        </is>
+      </c>
+      <c r="E25" s="47" t="inlineStr">
+        <is>
+          <t>core/services/inspection_release_store.py; core/services/inspection_maintenance.py
+tools/pcba_pilot.py; tools/production_preflight.py; tools/audit_cross_class_duplicates.py
+tests/conftest.py; models/Cable1/A/yolo/config.yaml
+docs/pilot/; docs/operations/; docs/manuals/</t>
+        </is>
+      </c>
+      <c r="F25" s="47" t="inlineStr">
+        <is>
+          <t>Tested code baseline SHA 8582a8b: PR run 32205343878 passed; workflow_dispatch 32205366029 passed, including the verified Windows executable. Configured blocking scoped mypy checks passed; this is not a whole-repo zero-findings claim. Local report-only, duplicate-filter, and audit regressions: 55 passed. Workspace exact-SHA CI also passed.</t>
+        </is>
+      </c>
+      <c r="G25" s="47" t="inlineStr">
+        <is>
+          <t>No current-head camera cycle, complete-shift/500-cycle suppress pilot, live company-sync/retention/rollback evidence, or named operational approvals are recorded. The production policy therefore remains report_only; suppress activation is blocked. Persisted fail-reason mapping for count/position lookup and no-detection color cases also remains incomplete.</t>
+        </is>
+      </c>
+      <c r="H25" s="47" t="inlineStr">
+        <is>
+          <t>Inference: 8582a8b
+Training: 41589fc
+Workspace: ee88317</t>
+        </is>
+      </c>
+      <c r="I25" s="47" t="inlineStr">
+        <is>
+          <t>Dio Wang</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:I23"/>
+  <autoFilter ref="A5:I25"/>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A3:I3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -3362,7 +3126,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.2"/>
   <cols>
     <col width="13" customWidth="1" style="41" min="1" max="1"/>
@@ -3380,14 +3144,14 @@
     <row r="1" ht="28" customHeight="1" s="41">
       <c r="A1" s="42" t="inlineStr">
         <is>
-          <t>Validation Evidence ? 2026-08-05 / 2026-08-13</t>
+          <t>Validation Evidence — 2026-08-05 through 2026-08-19</t>
         </is>
       </c>
     </row>
     <row r="2" ht="26" customHeight="1" s="41">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>Targeted regression only. Full commands are retained as comments on the Runner cells; results are not a field-acceptance certificate.</t>
+          <t>Commands and evidence links are retained in Runner-cell comments or linked CI logs where available; legacy rows with incomplete provenance are identified explicitly.</t>
         </is>
       </c>
     </row>
@@ -3444,10 +3208,8 @@
       </c>
     </row>
     <row r="5" ht="68" customHeight="1" s="41">
-      <c r="A5" s="47" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
+      <c r="A5" s="59" t="n">
+        <v>46239</v>
       </c>
       <c r="B5" s="47" t="inlineStr">
         <is>
@@ -3496,10 +3258,8 @@
       </c>
     </row>
     <row r="6" ht="68" customHeight="1" s="41">
-      <c r="A6" s="47" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
+      <c r="A6" s="59" t="n">
+        <v>46239</v>
       </c>
       <c r="B6" s="47" t="inlineStr">
         <is>
@@ -3548,10 +3308,8 @@
       </c>
     </row>
     <row r="7" ht="68" customHeight="1" s="41">
-      <c r="A7" s="47" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
+      <c r="A7" s="59" t="n">
+        <v>46239</v>
       </c>
       <c r="B7" s="47" t="inlineStr">
         <is>
@@ -3600,10 +3358,8 @@
       </c>
     </row>
     <row r="8" ht="68" customHeight="1" s="41">
-      <c r="A8" s="47" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
+      <c r="A8" s="59" t="n">
+        <v>46239</v>
       </c>
       <c r="B8" s="47" t="inlineStr">
         <is>
@@ -3652,10 +3408,8 @@
       </c>
     </row>
     <row r="9" ht="68" customHeight="1" s="41">
-      <c r="A9" s="47" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
+      <c r="A9" s="59" t="n">
+        <v>46239</v>
       </c>
       <c r="B9" s="47" t="inlineStr">
         <is>
@@ -3703,7 +3457,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="68" customHeight="1" s="41">
+    <row r="10" ht="82" customHeight="1" s="41">
       <c r="A10" s="47" t="inlineStr">
         <is>
           <t>Not recorded</t>
@@ -3747,15 +3501,13 @@
       <c r="I10" s="47" t="inlineStr"/>
       <c r="J10" s="47" t="inlineStr">
         <is>
-          <t>Do not infer field reliability, latency percentiles, or inspection accuracy from the automated tests above.</t>
+          <t>Report-only code integration does not certify field operation. A current-head camera cycle, a complete shift and at least 500 cycles, live sync/retention/rollback evidence, and named approvals remain NOT RECORDED; suppress activation is blocked.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="68" customHeight="1" s="41">
-      <c r="A11" s="47" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
+      <c r="A11" s="59" t="n">
+        <v>46239</v>
       </c>
       <c r="B11" s="47" t="inlineStr">
         <is>
@@ -3804,10 +3556,8 @@
       </c>
     </row>
     <row r="12" ht="68" customHeight="1" s="41">
-      <c r="A12" s="47" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
+      <c r="A12" s="59" t="n">
+        <v>46247</v>
       </c>
       <c r="B12" s="47" t="inlineStr">
         <is>
@@ -3855,11 +3605,9 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="68" customHeight="1" s="41">
-      <c r="A13" s="47" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
+    <row r="13" ht="88" customHeight="1" s="41">
+      <c r="A13" s="59" t="n">
+        <v>46247</v>
       </c>
       <c r="B13" s="47" t="inlineStr">
         <is>
@@ -3891,9 +3639,9 @@
           <t>Full inference suite</t>
         </is>
       </c>
-      <c r="H13" s="49" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+      <c r="H13" s="62" t="inlineStr">
+        <is>
+          <t>BLOCKED — HOST DISK CAPACITY</t>
         </is>
       </c>
       <c r="I13" s="47" t="inlineStr">
@@ -3903,18 +3651,168 @@
       </c>
       <c r="J13" s="47" t="inlineStr">
         <is>
-          <t>The 12 failures are test_result_handler disk-capacity guard trips (free 635-821 MiB against a 1024 MiB reserve), not defects in the release. An unmodified baseline reproduced the same 12 failures.</t>
+          <t>The 12 failures are test_result_handler disk-capacity guard trips (free 635-821 MiB against a 1024 MiB reserve), not newly introduced by the v1.1.0 change. Reproduction on an unmodified baseline does not rule out a pre-existing software defect. Historical run; superseded for current merge-readiness by the exact-SHA CI recorded on 2026-08-19, but retained as blocked historical evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="88" customHeight="1" s="41">
+      <c r="A14" s="59" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B14" s="47" t="inlineStr">
+        <is>
+          <t>yolo11_inference</t>
+        </is>
+      </c>
+      <c r="C14" s="47" t="inlineStr">
+        <is>
+          <t>3.10 / 3.11</t>
+        </is>
+      </c>
+      <c r="D14" s="47" t="inlineStr">
+        <is>
+          <t>2.4.1</t>
+        </is>
+      </c>
+      <c r="E14" s="47" t="inlineStr">
+        <is>
+          <t>GitHub Actions</t>
+        </is>
+      </c>
+      <c r="F14" s="47" t="inlineStr">
+        <is>
+          <t>CI / workflow_dispatch</t>
+        </is>
+      </c>
+      <c r="G14" s="47" t="inlineStr">
+        <is>
+          <t>Quality; Linux/Windows tests; coverage; package; verified Windows executable; report-only policy regression</t>
+        </is>
+      </c>
+      <c r="H14" s="49" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I14" s="47" t="inlineStr">
+        <is>
+          <t>All required jobs passed</t>
+        </is>
+      </c>
+      <c r="J14" s="47" t="inlineStr">
+        <is>
+          <t>Tested code baseline SHA 8582a8b. PR run 32205343878 and dispatch 32205366029 passed; local policy/filter/audit regression: 55 passed. Automated evidence only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="88" customHeight="1" s="41">
+      <c r="A15" s="59" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B15" s="47" t="inlineStr">
+        <is>
+          <t>Yolo11_auto_train</t>
+        </is>
+      </c>
+      <c r="C15" s="47" t="inlineStr">
+        <is>
+          <t>3.10 / 3.11</t>
+        </is>
+      </c>
+      <c r="D15" s="47" t="inlineStr">
+        <is>
+          <t>2.4.1</t>
+        </is>
+      </c>
+      <c r="E15" s="47" t="inlineStr">
+        <is>
+          <t>GitHub Actions</t>
+        </is>
+      </c>
+      <c r="F15" s="47" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="G15" s="47" t="inlineStr">
+        <is>
+          <t>Quality; Linux/Windows tests; coverage; package</t>
+        </is>
+      </c>
+      <c r="H15" s="49" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I15" s="47" t="inlineStr">
+        <is>
+          <t>All required jobs passed</t>
+        </is>
+      </c>
+      <c r="J15" s="47" t="inlineStr">
+        <is>
+          <t>Exact SHA 41589fc. Push run 32205326796 and PR run 32205329324 attempt 2 passed. Attempt 1 had one timing-only Windows heartbeat threshold failure; the same SHA passed on rerun.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="88" customHeight="1" s="41">
+      <c r="A16" s="59" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B16" s="47" t="inlineStr">
+        <is>
+          <t>Workspace integration</t>
+        </is>
+      </c>
+      <c r="C16" s="47" t="inlineStr">
+        <is>
+          <t>3.11</t>
+        </is>
+      </c>
+      <c r="D16" s="47" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E16" s="47" t="inlineStr">
+        <is>
+          <t>GitHub Actions / local</t>
+        </is>
+      </c>
+      <c r="F16" s="47" t="inlineStr">
+        <is>
+          <t>Workspace CI</t>
+        </is>
+      </c>
+      <c r="G16" s="47" t="inlineStr">
+        <is>
+          <t>Exact child SHAs; workspace validator; integration scripts; coverage</t>
+        </is>
+      </c>
+      <c r="H16" s="49" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I16" s="47" t="inlineStr">
+        <is>
+          <t>28 passed; 84.68% coverage</t>
+        </is>
+      </c>
+      <c r="J16" s="47" t="inlineStr">
+        <is>
+          <t>Pre-document integration baseline SHA ee88317. Workspace runs 32206682344 and 32206684956 passed, including the coherent exact-SHA child gate. Automated integration evidence only.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J11"/>
+  <autoFilter ref="A4:J16"/>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>